<commit_message>
feat: initial project structure without datasets
</commit_message>
<xml_diff>
--- a/EXAM_FORM1_RESULTS/EXAM_FORM1_19283.xlsx
+++ b/EXAM_FORM1_RESULTS/EXAM_FORM1_19283.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>07/05/2028</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>414</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -548,7 +548,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ile</t>
+          <t>Jnliew</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RIE LU</t>
+          <t>MCKEAN</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -582,7 +582,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>G04E</t>
+          <t>G04D</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>12835</v>
+        <v>19283</v>
       </c>
     </row>
     <row r="18">

</xml_diff>